<commit_message>
Show only ticker symbol in A3 Name of entity column
A3 column C now uses the IBKR symbol (e.g. NOVd, AAPL) instead of
legal name + ticker + qty. Regenerated Ray Stephanos AY2026-27 workbook.

Co-authored-by: yashjain-a11y <yashjain-a11y@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/output/Foreign_Assets_Schedule_FA_Ray_G_Stephanos_AY2026-27.xlsx
+++ b/output/Foreign_Assets_Schedule_FA_Ray_G_Stephanos_AY2026-27.xlsx
@@ -4579,7 +4579,7 @@
   <cols>
     <col width="48" customWidth="1" min="1" max="1"/>
     <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="48" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
     <col width="48" customWidth="1" min="4" max="4"/>
     <col width="10" customWidth="1" min="5" max="5"/>
     <col width="48" customWidth="1" min="6" max="6"/>
@@ -4710,7 +4710,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Xiaomi Corp - Class B  [Ticker: 1810]  Qty: 200</t>
+          <t>1810</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -4756,7 +4756,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>COSCO Shipping Holdings Co - H  [Ticker: 1919]  Qty: 500</t>
+          <t>1919</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -4802,7 +4802,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>ChinaAMC Hang Seng Biotech ETF  [Ticker: 3069]  Qty: 600</t>
+          <t>3069</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -4848,7 +4848,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>ChinaAMC Hang Seng TECH Index ETF  [Ticker: 3088]  Qty: 1000</t>
+          <t>3088</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -4894,7 +4894,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>ChinaAMC CSI 300 Index ETF  [Ticker: 3188]  Qty: 200</t>
+          <t>3188</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -4940,7 +4940,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Global X HSCEI Covered Call ETF  [Ticker: 3416]  Qty: 1000</t>
+          <t>3416</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -4986,7 +4986,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Daiichi Sankyo Co Ltd  [Ticker: 4568.T]  Qty: 100</t>
+          <t>4568.T</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -5036,7 +5036,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Apple Inc - Common Stock  [Ticker: AAPL]  Qty: 7</t>
+          <t>AAPL</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -5086,7 +5086,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>iShares MSCI All Country Asia ex Japan ETF  [Ticker: AAXJ]  Qty: 8</t>
+          <t>AAXJ</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -5136,7 +5136,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Global X Artificial Intelligence &amp; Technology ETF  [Ticker: AIQ]  Qty: 36</t>
+          <t>AIQ</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -5186,7 +5186,7 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>AIR  [Ticker: AIR]  Qty: 0</t>
+          <t>AIR</t>
         </is>
       </c>
       <c r="D15" t="inlineStr"/>
@@ -5228,7 +5228,7 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Airbus SE  [Ticker: AIRd]  Qty: 10</t>
+          <t>AIRd</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -5278,7 +5278,7 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Advanced Micro Devices Inc  [Ticker: AMD]  Qty: 1.2</t>
+          <t>AMD</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -5328,7 +5328,7 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Advanced Micro Devices Inc  [Ticker: AMD]  Qty: 9</t>
+          <t>AMD</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -5378,7 +5378,7 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Amazon.com Inc  [Ticker: AMZN]  Qty: 6</t>
+          <t>AMZN</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -5428,7 +5428,7 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>ASML Holding NV - NY Registered Shares  [Ticker: ASML]  Qty: 6</t>
+          <t>ASML</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
@@ -5478,7 +5478,7 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>ASML Holding NV - NY Registered Shares  [Ticker: ASML]  Qty: 3</t>
+          <t>ASML</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
@@ -5528,7 +5528,7 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Broadcom Inc  [Ticker: AVGO]  Qty: 9</t>
+          <t>AVGO</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
@@ -5578,7 +5578,7 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Bank of America Corp  [Ticker: BAC]  Qty: 60</t>
+          <t>BAC</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
@@ -5628,7 +5628,7 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Blue Bird Corp  [Ticker: BLBD]  Qty: 60</t>
+          <t>BLBD</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
@@ -5678,7 +5678,7 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Global X Robotics &amp; Artificial Intelligence ETF  [Ticker: BOTZ]  Qty: 24</t>
+          <t>BOTZ</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
@@ -5728,7 +5728,7 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>British American Tobacco plc - Sponsored ADR  [Ticker: BTI]  Qty: 33</t>
+          <t>BTI</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
@@ -5778,7 +5778,7 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Blackstone Inc  [Ticker: BX]  Qty: 12</t>
+          <t>BX</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
@@ -5828,7 +5828,7 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>BYD Co Ltd - Unsponsored ADR  [Ticker: BYDDY]  Qty: 42</t>
+          <t>BYDDY</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
@@ -5878,7 +5878,7 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Caterpillar Inc  [Ticker: CAT]  Qty: 3</t>
+          <t>CAT</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
@@ -5928,7 +5928,7 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Caterpillar Inc  [Ticker: CAT]  Qty: 6</t>
+          <t>CAT</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
@@ -5978,7 +5978,7 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>ClearPoint Neuro Inc  [Ticker: CLPT]  Qty: 42</t>
+          <t>CLPT</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
@@ -6028,7 +6028,7 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Coupang Inc (Delaware) - Class A  [Ticker: CPNG]  Qty: 50</t>
+          <t>CPNG</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
@@ -6078,7 +6078,7 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Circle Internet Group Inc  [Ticker: CRCL]  Qty: 1</t>
+          <t>CRCL</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
@@ -6128,7 +6128,7 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Circle Internet Group Inc  [Ticker: CRCL]  Qty: 19</t>
+          <t>CRCL</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
@@ -6178,7 +6178,7 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Circle Internet Group Inc  [Ticker: CRCL]  Qty: 30.0554</t>
+          <t>CRCL</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
@@ -6228,7 +6228,7 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Circle Internet Group Inc  [Ticker: CRCL]  Qty: 10</t>
+          <t>CRCL</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
@@ -6278,7 +6278,7 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Cisco Systems Inc  [Ticker: CSCO]  Qty: 20</t>
+          <t>CSCO</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
@@ -6328,7 +6328,7 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Deutsche Bank AG - Registered Shares  [Ticker: DB]  Qty: 33</t>
+          <t>DB</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
@@ -6378,7 +6378,7 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Duolingo Inc  [Ticker: DUOL]  Qty: 3</t>
+          <t>DUOL</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
@@ -6428,7 +6428,7 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Duolingo Inc  [Ticker: DUOL]  Qty: 6</t>
+          <t>DUOL</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
@@ -6478,7 +6478,7 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>WisdomTree Japan Hedged Equity Fund  [Ticker: DXJ]  Qty: 6</t>
+          <t>DXJ</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
@@ -6528,7 +6528,7 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>iShares MSCI Emerging Markets ex China ETF  [Ticker: EMXC]  Qty: 9</t>
+          <t>EMXC</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
@@ -6578,7 +6578,7 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>General Dynamics Corp  [Ticker: GD]  Qty: 6</t>
+          <t>GD</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
@@ -6628,7 +6628,7 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>GE Aerospace / General Electric  [Ticker: GE]  Qty: 3</t>
+          <t>GE</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
@@ -6678,7 +6678,7 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>SPDR Gold Shares (World Gold Trust)  [Ticker: GLD]  Qty: 10</t>
+          <t>GLD</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
@@ -6728,7 +6728,7 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Hyundai Motor Co - Reg S GDR  [Ticker: HYU]  Qty: 24</t>
+          <t>HYU</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
@@ -6778,7 +6778,7 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>International Business Machines Corp  [Ticker: IBM]  Qty: 5</t>
+          <t>IBM</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
@@ -6828,7 +6828,7 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>iShares Global Clean Energy ETF  [Ticker: ICLN]  Qty: 50</t>
+          <t>ICLN</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
@@ -6878,7 +6878,7 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>Invesco AI and Next Gen Software ETF  [Ticker: IGPT]  Qty: 33</t>
+          <t>IGPT</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
@@ -6928,7 +6928,7 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>Intel Corp  [Ticker: INTC]  Qty: 72</t>
+          <t>INTC</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
@@ -6978,7 +6978,7 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>iShares Russell Mid-Cap ETF  [Ticker: IWR]  Qty: 10</t>
+          <t>IWR</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
@@ -7028,7 +7028,7 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>Eli Lilly &amp; Company  [Ticker: LLY]  Qty: 6</t>
+          <t>LLY</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
@@ -7078,7 +7078,7 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>Eli Lilly &amp; Company  [Ticker: LLY]  Qty: 3.5</t>
+          <t>LLY</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
@@ -7128,7 +7128,7 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>Lam Research Corp  [Ticker: LRCX]  Qty: 90</t>
+          <t>LRCX</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
@@ -7178,7 +7178,7 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>Lam Research Corp  [Ticker: LRCX]  Qty: 10</t>
+          <t>LRCX</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
@@ -7228,7 +7228,7 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>iShares MSCI China ETF  [Ticker: MCHI]  Qty: 27</t>
+          <t>MCHI</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
@@ -7278,7 +7278,7 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>Meta Platforms Inc - Class A  [Ticker: META]  Qty: 2</t>
+          <t>META</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
@@ -7328,7 +7328,7 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>Microsoft Corp  [Ticker: MSFT]  Qty: 6</t>
+          <t>MSFT</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
@@ -7378,7 +7378,7 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>Nebius Group NV  [Ticker: NBIS]  Qty: 15</t>
+          <t>NBIS</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
@@ -7428,7 +7428,7 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>Netflix Inc  [Ticker: NFLX]  Qty: 2.4</t>
+          <t>NFLX</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
@@ -7478,7 +7478,7 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>Netflix Inc  [Ticker: NFLX]  Qty: 10</t>
+          <t>NFLX</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
@@ -7528,7 +7528,7 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>NOV  [Ticker: NOV]  Qty: 0</t>
+          <t>NOV</t>
         </is>
       </c>
       <c r="D62" t="inlineStr"/>
@@ -7570,7 +7570,7 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>Novo Nordisk A/S - B Shares  [Ticker: NOVd]  Qty: 30</t>
+          <t>NOVd</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
@@ -7620,7 +7620,7 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>Novo Nordisk A/S - B Shares  [Ticker: NOVd]  Qty: 55</t>
+          <t>NOVd</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
@@ -7670,7 +7670,7 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>NVIDIA Corp  [Ticker: NVDA]  Qty: 4.2</t>
+          <t>NVDA</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
@@ -7720,7 +7720,7 @@
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>NVIDIA Corp  [Ticker: NVDA]  Qty: 12</t>
+          <t>NVDA</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
@@ -7770,7 +7770,7 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>Oracle Corp  [Ticker: ORCL]  Qty: 5</t>
+          <t>ORCL</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
@@ -7820,7 +7820,7 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>Invesco QQQ Trust Series 1  [Ticker: QQQ]  Qty: 2</t>
+          <t>QQQ</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
@@ -7870,7 +7870,7 @@
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>Shell plc  [Ticker: R6C0d]  Qty: 42</t>
+          <t>R6C0d</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
@@ -7920,7 +7920,7 @@
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>Rubrik Inc - Class A  [Ticker: RBRK]  Qty: 17</t>
+          <t>RBRK</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
@@ -7970,7 +7970,7 @@
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>Regeneron Pharmaceuticals Inc  [Ticker: REGN]  Qty: 3</t>
+          <t>REGN</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
@@ -8020,7 +8020,7 @@
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>Rio Tinto plc - Sponsored ADR  [Ticker: RIO]  Qty: 9</t>
+          <t>RIO</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
@@ -8070,7 +8070,7 @@
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>RTX Corp  [Ticker: RTX]  Qty: 30</t>
+          <t>RTX</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
@@ -8120,7 +8120,7 @@
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>iShares MSCI Australia UCITS ETF  [Ticker: SAUS]  Qty: 6</t>
+          <t>SAUS</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
@@ -8170,7 +8170,7 @@
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>Siemens AG - Registered  [Ticker: SIEd]  Qty: 20</t>
+          <t>SIEd</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
@@ -8220,7 +8220,7 @@
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>Snowflake Inc  [Ticker: SNOW]  Qty: 8</t>
+          <t>SNOW</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
@@ -8270,7 +8270,7 @@
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>Target Corp  [Ticker: TGT]  Qty: 6</t>
+          <t>TGT</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
@@ -8320,7 +8320,7 @@
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>Target Corp  [Ticker: TGT]  Qty: 20</t>
+          <t>TGT</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
@@ -8370,7 +8370,7 @@
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>iShares TIPS Bond ETF  [Ticker: TIP]  Qty: 60</t>
+          <t>TIP</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
@@ -8420,7 +8420,7 @@
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>Tesla Inc  [Ticker: TSLA]  Qty: 10</t>
+          <t>TSLA</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
@@ -8470,7 +8470,7 @@
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>Taiwan Semiconductor Manufacturing Co - Sponsored ADR  [Ticker: TSM]  Qty: 6</t>
+          <t>TSM</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
@@ -8520,7 +8520,7 @@
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>Viking Therapeutics Inc  [Ticker: VKTX]  Qty: 33</t>
+          <t>VKTX</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
@@ -8570,7 +8570,7 @@
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>Vanguard Total World Stock ETF  [Ticker: VT]  Qty: 9</t>
+          <t>VT</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
@@ -8620,7 +8620,7 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>Vanguard Value ETF  [Ticker: VTV]  Qty: 6</t>
+          <t>VTV</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
@@ -8670,7 +8670,7 @@
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>WisdomTree Cybersecurity UCITS ETF  [Ticker: WCBR]  Qty: 75</t>
+          <t>WCBR</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
@@ -8720,7 +8720,7 @@
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>Wells Fargo &amp; Company  [Ticker: WFC]  Qty: 50</t>
+          <t>WFC</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">

</xml_diff>

<commit_message>
Add Schedule FA workbook for Puneet Kohli (U17334752)
Generate AY2026-27 FA/CG/dividends output matching Ray format (A3 Col C =
symbol only). Handles FOP stock transfers as FIFO acquisitions using IBKR
cost basis. Synthesizes CY2025 annual from FY statements + YE MSFT close
when Annual Activity Statement is not furnished. Fixes account-info
overwrite bug in A2/Notes.

Co-authored-by: yashjain-a11y <yashjain-a11y@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/output/Foreign_Assets_Schedule_FA_Ray_G_Stephanos_AY2026-27.xlsx
+++ b/output/Foreign_Assets_Schedule_FA_Ray_G_Stephanos_AY2026-27.xlsx
@@ -4168,7 +4168,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B34"/>
+  <dimension ref="A1:B35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="48" customWidth="1" min="1" max="1"/>
@@ -4188,6 +4188,11 @@
           <t>Assessee</t>
         </is>
       </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Ray G Stephanos</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -4197,7 +4202,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>None — Interactive Brokers LLC (Advisor Client; Advisor: None)</t>
+          <t>U15124027 — Interactive Brokers LLC (Advisor Client; Advisor: Financial Hospital Advisory LLP)</t>
         </is>
       </c>
     </row>
@@ -4207,6 +4212,11 @@
           <t>Customer type</t>
         </is>
       </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Individual</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -4214,6 +4224,11 @@
           <t>Base currency</t>
         </is>
       </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -4463,7 +4478,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Applicable — see sheet; opening date 06-Sep-2024 (first funding)</t>
+          <t>Applicable — see sheet; opening: 2024-09-06 (first funding / inbound transfer per IBKR)</t>
         </is>
       </c>
     </row>
@@ -4482,82 +4497,94 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>A3 vs CG</t>
+          <t>A3 Col C (Name of entity)</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Sold lots: A3 Initial = CG Cost (INR), A3 Sale = CG Sale (INR), same Rule 115/EUR FX. Multiple buys (e.g. NOVd 21-Mar &amp; 21-Aug) appear as separate A3 rows.</t>
+          <t>Symbol only (e.g. NOVd, AAPL). Legal name / address remain in Address &amp; Nature columns.</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>ADR country practice</t>
+          <t>A3 vs CG</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Underlying issuer country used for ADRs/GDRs (ASML NL, BTI UK, TSM TW, BYDDY CN, HYU KR, RIO UK)</t>
+          <t>Sold lots: A3 Initial = CG Cost (INR), A3 Sale = CG Sale (INR), same Rule 115/EUR FX. Multiple buys (e.g. NOVd 21-Mar &amp; 21-Aug) appear as separate A3 rows.</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>CPNG</t>
+          <t>ADR country practice</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>USA (Delaware corporation, NYSE) despite Korea operations</t>
+          <t>Underlying issuer country used for ADRs/GDRs (ASML NL, BTI UK, TSM TW, BYDDY CN, HYU KR, RIO UK)</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>NFLX split</t>
+          <t>CPNG</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>10-for-1 split on 14/17-Nov-2025 reflected in FIFO</t>
+          <t>USA (Delaware corporation, NYSE) despite Korea operations</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>LRCX split</t>
+          <t>NFLX split</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>10-for-1 split on 02/03-Oct-2024 reflected in FIFO (bought 1 pre-split → 10)</t>
+          <t>10-for-1 split on 14/17-Nov-2025 reflected in FIFO</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>HYU</t>
+          <t>LRCX split</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Cash merger acquisition Jul-2025 — sale proceeds USD 1,339.02 reported as redemption proceeds</t>
+          <t>10-for-1 split on 02/03-Oct-2024 reflected in FIFO (bought 1 pre-split → 10)</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
+          <t>HYU</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>Cash merger acquisition Jul-2025 — sale proceeds USD 1,339.02 reported as redemption proceeds</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
           <t>Action required</t>
         </is>
       </c>
-      <c r="B34" t="inlineStr">
+      <c r="B35" t="inlineStr">
         <is>
           <t>1) Confirm exact SBI TT Buy card rates; 2) Obtain PortfolioAnalyst for true peak NAV; 3) Map withholding to Schedule FSI/TR under DTAA.</t>
         </is>
@@ -13318,7 +13345,7 @@
     <col width="31" customWidth="1" min="5" max="5"/>
     <col width="31" customWidth="1" min="6" max="6"/>
     <col width="34" customWidth="1" min="7" max="7"/>
-    <col width="46" customWidth="1" min="8" max="8"/>
+    <col width="48" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -13381,7 +13408,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Interactive Brokers LLC (Clearing Broker), Advisor Client via Interactive Brokers (India) / Investment Advisor: </t>
+          <t>Interactive Brokers LLC (Clearing Broker), Advisor Client via Interactive Brokers (India) / Investment Advisor: Financial Hospital Advisory LLP</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -13394,7 +13421,11 @@
           <t>06830</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr"/>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>U15124027</t>
+        </is>
+      </c>
       <c r="G3" t="inlineStr">
         <is>
           <t>Owner - Sole beneficial owner</t>
@@ -13402,7 +13433,7 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>2024-09-06 (first funding per IBKR deposits)</t>
+          <t>2024-09-06 (first funding / inbound transfer per IBKR)</t>
         </is>
       </c>
     </row>
@@ -13486,7 +13517,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Account: IBKR None — None (Individual, USD base, Cash).</t>
+          <t>Account: IBKR U15124027 — Ray G Stephanos (Individual, USD base, Cash).</t>
         </is>
       </c>
     </row>

</xml_diff>